<commit_message>
Add ticket generation, admin chat improvements, and sales chart filters.
Rebrand live support to ticket submission, enhance admin customer chat with unread badges and thread management, fix dashboard loading, and add filtered sales charts with shared dropdown styling.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sheet_template.xlsx
+++ b/sheet_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Intern_project\E-Commerce_website\drone-e-commerce-platform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9096AAC-74B2-48A3-AFB3-42ADEED0F426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C1C68E-890A-4A02-B400-10E2D154AD8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,9 +33,6 @@
     <t>Sl.NO</t>
   </si>
   <si>
-    <t>ID</t>
-  </si>
-  <si>
     <t>QTY</t>
   </si>
   <si>
@@ -43,6 +40,9 @@
   </si>
   <si>
     <t>HDS-GRD-X500-002</t>
+  </si>
+  <si>
+    <t>Model Number</t>
   </si>
 </sst>
 </file>
@@ -386,10 +386,10 @@
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:4">
@@ -397,7 +397,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3" s="1">
         <v>10</v>
@@ -408,7 +408,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" s="1">
         <v>20</v>

</xml_diff>